<commit_message>
docs: update AMR roadmap (xlsx + ods copy)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/document/AMR_Roadmap.xlsx
+++ b/document/AMR_Roadmap.xlsx
@@ -131,25 +131,25 @@
     <t xml:space="preserve">2</t>
   </si>
   <si>
+    <t xml:space="preserve">P1-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calibrate wheel_sep (track width) ด้วยการหมุนอยู่กับที่</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หมุน 360°/720° CW และ CCW ×5 รอบ วัดมุมจริงด้วยเส้นอ้างอิง/LiDAR; wheel_sep_true = nominal × commanded / actual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">มุมสะสม error &lt;1° ต่อ 360°; CW กับ CCW ต่างกัน &lt;1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">calib_rotate_node.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
     <t xml:space="preserve">ยังไม่เริ่ม</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P1-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calibrate wheel_sep (track width) ด้วยการหมุนอยู่กับที่</t>
-  </si>
-  <si>
-    <t xml:space="preserve">หมุน 360°/720° CW และ CCW ×5 รอบ วัดมุมจริงด้วยเส้นอ้างอิง/LiDAR; wheel_sep_true = nominal × commanded / actual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">มุมสะสม error &lt;1° ต่อ 360°; CW กับ CCW ต่างกัน &lt;1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">calib_rotate_node.py</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
   </si>
   <si>
     <t xml:space="preserve">ทดสอบความเร็วต่ำ พื้นที่โล่ง ตรวจ E-stop ก่อน</t>
@@ -806,13 +806,12 @@
     <numFmt numFmtId="165" formatCode="0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -834,14 +833,12 @@
       <sz val="14"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
       <sz val="9"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -849,20 +846,12 @@
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -870,14 +859,12 @@
       <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -960,6 +947,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -968,43 +959,39 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1017,7 +1004,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1063,6 +1050,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFF7F7F7"/>
+          <bgColor rgb="FF272727"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FF0000FF"/>
         </patternFill>
       </fill>
@@ -1082,6 +1077,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
@@ -1089,6 +1090,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
@@ -1096,6 +1103,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
@@ -1103,6 +1116,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFBDD7EE"/>
@@ -1110,6 +1129,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFF8CBAD"/>
@@ -1117,6 +1142,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFF2CC"/>
@@ -1124,6 +1155,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFE2EFDA"/>
@@ -1204,7 +1241,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L43"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
@@ -1220,7 +1257,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="36"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1241,7 +1278,7 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1279,7 +1316,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>14</v>
       </c>
@@ -1347,7 +1384,7 @@
       <c r="K6" s="5"/>
       <c r="L6" s="4"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
         <v>29</v>
       </c>
@@ -1376,48 +1413,48 @@
         <v>1</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K7" s="5"/>
       <c r="L7" s="4"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>20</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K8" s="5"/>
       <c r="L8" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
         <v>43</v>
       </c>
@@ -1446,14 +1483,14 @@
         <v>0.5</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K9" s="5"/>
       <c r="L9" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
         <v>50</v>
       </c>
@@ -1482,12 +1519,12 @@
         <v>2</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K10" s="5"/>
       <c r="L10" s="4"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
         <v>57</v>
       </c>
@@ -1516,12 +1553,12 @@
         <v>0.5</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K11" s="5"/>
       <c r="L11" s="4"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
         <v>63</v>
       </c>
@@ -1550,12 +1587,12 @@
         <v>1</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K12" s="5"/>
       <c r="L12" s="4"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
         <v>69</v>
       </c>
@@ -1584,14 +1621,14 @@
         <v>0.25</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K13" s="5"/>
       <c r="L13" s="4" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
         <v>75</v>
       </c>
@@ -1614,18 +1651,18 @@
         <v>55</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K14" s="5"/>
       <c r="L14" s="4"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
         <v>80</v>
       </c>
@@ -1654,14 +1691,14 @@
         <v>1</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K15" s="5"/>
       <c r="L15" s="4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
         <v>87</v>
       </c>
@@ -1690,12 +1727,12 @@
         <v>1</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K16" s="5"/>
       <c r="L16" s="4"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
         <v>94</v>
       </c>
@@ -1724,12 +1761,12 @@
         <v>2</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K17" s="5"/>
       <c r="L17" s="4"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
         <v>99</v>
       </c>
@@ -1758,14 +1795,14 @@
         <v>1</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K18" s="5"/>
       <c r="L18" s="6" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
         <v>105</v>
       </c>
@@ -1794,12 +1831,12 @@
         <v>1</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K19" s="5"/>
       <c r="L19" s="4"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
         <v>112</v>
       </c>
@@ -1828,12 +1865,12 @@
         <v>1</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K20" s="5"/>
       <c r="L20" s="4"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
         <v>117</v>
       </c>
@@ -1862,12 +1899,12 @@
         <v>2</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K21" s="5"/>
       <c r="L21" s="4"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
         <v>122</v>
       </c>
@@ -1890,18 +1927,18 @@
         <v>55</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I22" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K22" s="5"/>
       <c r="L22" s="4"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
         <v>127</v>
       </c>
@@ -1930,12 +1967,12 @@
         <v>1</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K23" s="5"/>
       <c r="L23" s="4"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
         <v>134</v>
       </c>
@@ -1964,14 +2001,14 @@
         <v>2</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K24" s="5"/>
       <c r="L24" s="6" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
         <v>140</v>
       </c>
@@ -2000,12 +2037,12 @@
         <v>3</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K25" s="5"/>
       <c r="L25" s="4"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
         <v>144</v>
       </c>
@@ -2028,18 +2065,18 @@
         <v>55</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I26" s="5" t="n">
         <v>2</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K26" s="5"/>
       <c r="L26" s="4"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
         <v>149</v>
       </c>
@@ -2068,12 +2105,12 @@
         <v>3</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K27" s="5"/>
       <c r="L27" s="4"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
         <v>154</v>
       </c>
@@ -2100,14 +2137,14 @@
         <v>2</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K28" s="5"/>
       <c r="L28" s="4" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
         <v>161</v>
       </c>
@@ -2136,14 +2173,14 @@
         <v>2</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K29" s="5"/>
       <c r="L29" s="6" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
         <v>167</v>
       </c>
@@ -2172,14 +2209,14 @@
         <v>3</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K30" s="5"/>
       <c r="L30" s="6" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
         <v>173</v>
       </c>
@@ -2208,12 +2245,12 @@
         <v>1</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K31" s="5"/>
       <c r="L31" s="4"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
         <v>177</v>
       </c>
@@ -2240,12 +2277,12 @@
         <v>2</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K32" s="5"/>
       <c r="L32" s="4"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
         <v>182</v>
       </c>
@@ -2274,14 +2311,14 @@
         <v>2</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K33" s="5"/>
       <c r="L33" s="6" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
         <v>188</v>
       </c>
@@ -2310,12 +2347,12 @@
         <v>1</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K34" s="5"/>
       <c r="L34" s="4"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
         <v>195</v>
       </c>
@@ -2344,14 +2381,14 @@
         <v>2</v>
       </c>
       <c r="J35" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K35" s="5"/>
       <c r="L35" s="4" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
         <v>201</v>
       </c>
@@ -2380,14 +2417,14 @@
         <v>4</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K36" s="5"/>
       <c r="L36" s="4" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
         <v>207</v>
       </c>
@@ -2414,12 +2451,12 @@
         <v>2</v>
       </c>
       <c r="J37" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K37" s="5"/>
       <c r="L37" s="4"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
         <v>212</v>
       </c>
@@ -2448,12 +2485,12 @@
         <v>1</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K38" s="5"/>
       <c r="L38" s="4"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
         <v>217</v>
       </c>
@@ -2480,14 +2517,14 @@
         <v>5</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K39" s="5"/>
       <c r="L39" s="4" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
         <v>223</v>
       </c>
@@ -2516,12 +2553,12 @@
         <v>10</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K40" s="5"/>
       <c r="L40" s="4"/>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
         <v>230</v>
       </c>
@@ -2550,12 +2587,12 @@
         <v>3</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K41" s="5"/>
       <c r="L41" s="4"/>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
         <v>235</v>
       </c>
@@ -2584,12 +2621,12 @@
         <v>1</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K42" s="5"/>
       <c r="L42" s="4"/>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
         <v>240</v>
       </c>
@@ -2616,7 +2653,7 @@
         <v>1</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K43" s="5"/>
       <c r="L43" s="4"/>
@@ -2627,37 +2664,37 @@
     <mergeCell ref="A2:L2"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J43">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>"เสร็จ"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>"กำลังทำ"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>"ติดปัญหา"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"รอตรวจ"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:G43">
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"สูง"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"กลาง"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"ต่ำ"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J43" type="list">
-      <formula1>"ยังไม่เริ่ม,กำลังทำ,รอตรวจ,เสร็จ,ติดปัญหา"</formula1>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G43" type="list">
+      <formula1>"สูง,กลาง,ต่ำ"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G43" type="list">
-      <formula1>"สูง,กลาง,ต่ำ"</formula1>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J43" type="list">
+      <formula1>"ยังไม่เริ่ม,กำลังทำ,รอตรวจ,เสร็จ,ติดปัญหา"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2678,18 +2715,18 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>3</v>
       </c>
@@ -2715,7 +2752,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
         <v>15</v>
       </c>
@@ -2725,7 +2762,7 @@
       </c>
       <c r="C4" s="8" t="n">
         <f aca="false">COUNTIFS(Roadmap!$B$5:$B$43,A4,Roadmap!$J$5:$J$43,"เสร็จ")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="8" t="n">
         <f aca="false">COUNTIFS(Roadmap!$B$5:$B$43,A4,Roadmap!$J$5:$J$43,"กำลังทำ")</f>
@@ -2737,7 +2774,7 @@
       </c>
       <c r="F4" s="9" t="n">
         <f aca="false">IF(B4=0,0,C4/B4)</f>
-        <v>0.333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="G4" s="10" t="n">
         <f aca="false">SUMIFS(Roadmap!$I$5:$I$43,Roadmap!$B$5:$B$43,A4)</f>
@@ -2745,10 +2782,10 @@
       </c>
       <c r="H4" s="10" t="n">
         <f aca="false">G4-SUMIFS(Roadmap!$I$5:$I$43,Roadmap!$B$5:$B$43,A4,Roadmap!$J$5:$J$43,"เสร็จ")</f>
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
         <v>58</v>
       </c>
@@ -2758,7 +2795,7 @@
       </c>
       <c r="C5" s="8" t="n">
         <f aca="false">COUNTIFS(Roadmap!$B$5:$B$43,A5,Roadmap!$J$5:$J$43,"เสร็จ")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D5" s="8" t="n">
         <f aca="false">COUNTIFS(Roadmap!$B$5:$B$43,A5,Roadmap!$J$5:$J$43,"กำลังทำ")</f>
@@ -2770,7 +2807,7 @@
       </c>
       <c r="F5" s="9" t="n">
         <f aca="false">IF(B5=0,0,C5/B5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="10" t="n">
         <f aca="false">SUMIFS(Roadmap!$I$5:$I$43,Roadmap!$B$5:$B$43,A5)</f>
@@ -2778,10 +2815,10 @@
       </c>
       <c r="H5" s="10" t="n">
         <f aca="false">G5-SUMIFS(Roadmap!$I$5:$I$43,Roadmap!$B$5:$B$43,A5,Roadmap!$J$5:$J$43,"เสร็จ")</f>
-        <v>3.75</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
         <v>88</v>
       </c>
@@ -2791,7 +2828,7 @@
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">COUNTIFS(Roadmap!$B$5:$B$43,A6,Roadmap!$J$5:$J$43,"เสร็จ")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="8" t="n">
         <f aca="false">COUNTIFS(Roadmap!$B$5:$B$43,A6,Roadmap!$J$5:$J$43,"กำลังทำ")</f>
@@ -2803,7 +2840,7 @@
       </c>
       <c r="F6" s="9" t="n">
         <f aca="false">IF(B6=0,0,C6/B6)</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="G6" s="10" t="n">
         <f aca="false">SUMIFS(Roadmap!$I$5:$I$43,Roadmap!$B$5:$B$43,A6)</f>
@@ -2811,10 +2848,10 @@
       </c>
       <c r="H6" s="10" t="n">
         <f aca="false">G6-SUMIFS(Roadmap!$I$5:$I$43,Roadmap!$B$5:$B$43,A6,Roadmap!$J$5:$J$43,"เสร็จ")</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
         <v>106</v>
       </c>
@@ -2847,7 +2884,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
         <v>128</v>
       </c>
@@ -2880,7 +2917,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
         <v>155</v>
       </c>
@@ -2913,7 +2950,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
         <v>189</v>
       </c>
@@ -2946,7 +2983,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
         <v>224</v>
       </c>
@@ -2979,7 +3016,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
         <v>252</v>
       </c>
@@ -2989,7 +3026,7 @@
       </c>
       <c r="C12" s="11" t="n">
         <f aca="false">SUM(C4:C11)</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D12" s="11" t="n">
         <f aca="false">SUM(D4:D11)</f>
@@ -3001,7 +3038,7 @@
       </c>
       <c r="F12" s="12" t="n">
         <f aca="false">IF(B12=0,0,C12/B12)</f>
-        <v>0.0512820512820513</v>
+        <v>0.230769230769231</v>
       </c>
       <c r="G12" s="13" t="n">
         <f aca="false">SUM(G4:G11)</f>
@@ -3009,25 +3046,25 @@
       </c>
       <c r="H12" s="13" t="n">
         <f aca="false">SUM(H4:H11)</f>
-        <v>70.25</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>64.5</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
         <v>256</v>
       </c>
@@ -3042,7 +3079,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{604A5DDA-5610-44D2-A4ED-D136F8BACF7E}</x14:id>
+          <x14:id>{BAA7BF77-4BFD-419F-B942-EFA43116B591}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3058,7 +3095,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{604A5DDA-5610-44D2-A4ED-D136F8BACF7E}">
+          <x14:cfRule type="dataBar" id="{BAA7BF77-4BFD-419F-B942-EFA43116B591}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>